<commit_message>
feat: add bag item selling
</commit_message>
<xml_diff>
--- a/Design/Excel/Localization.xlsx
+++ b/Design/Excel/Localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B622675-4911-4639-BE9B-462FBB374EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F01662-E3E1-4E9E-B532-8AEA4B0230F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="250">
   <si>
     <t>##</t>
   </si>
@@ -1634,6 +1634,14 @@
   </si>
   <si>
     <t>三火球</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bag_Sell</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>卖出</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -2098,7 +2106,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="2" max="2" width="23.33203125" customWidth="1"/>
@@ -2917,6 +2925,14 @@
       </c>
       <c r="C68" s="2" t="s">
         <v>196</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3">
+      <c r="B69" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>